<commit_message>
feat(linked-list): add LC 92 Reverse Linked List II & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{349F7476-C2CB-4A13-9308-1550511DFB6D}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{865CC496-5BDB-4B00-9B48-2753F5ACC996}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2831,7 +2831,9 @@
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" ht="14.4">
-      <c r="A62" s="6"/>
+      <c r="A62" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B62" s="9" t="s">
         <v>119</v>
       </c>

</xml_diff>

<commit_message>
feat(linked-list): add LC 24 Swap Nodes in Pairs & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{865CC496-5BDB-4B00-9B48-2753F5ACC996}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F95323BD-FBF0-45F7-A8E6-E5FA3CD5A77A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2844,7 +2844,9 @@
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="14.4">
-      <c r="A63" s="6"/>
+      <c r="A63" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B63" s="9" t="s">
         <v>121</v>
       </c>

</xml_diff>

<commit_message>
feat(linked-list): add LC 25 Reverse Nodes in k-Group & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F95323BD-FBF0-45F7-A8E6-E5FA3CD5A77A}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86882A68-6C38-44A3-8447-E0DC5AE4D46E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2857,7 +2857,9 @@
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="14.4">
-      <c r="A64" s="6"/>
+      <c r="A64" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B64" s="9" t="s">
         <v>123</v>
       </c>

</xml_diff>

<commit_message>
feat(linked-list): add LC 2074 Reverse Nodes in Even Length Groups & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86882A68-6C38-44A3-8447-E0DC5AE4D46E}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9F511F9-E1EF-4531-937A-1BBAC6A99C55}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2870,7 +2870,9 @@
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="14.4">
-      <c r="A65" s="6"/>
+      <c r="A65" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B65" s="6" t="s">
         <v>125</v>
       </c>

</xml_diff>

<commit_message>
feat(linked-list): add LC 61 Rotate List & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9F511F9-E1EF-4531-937A-1BBAC6A99C55}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9404AF28-04A8-4EF3-93F7-455BF9EA77A8}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2883,7 +2883,9 @@
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="14.4">
-      <c r="A66" s="6"/>
+      <c r="A66" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B66" s="9" t="s">
         <v>127</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): create Stack directory, add LC 1047 Remove All Adjacent Duplicates In String & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9404AF28-04A8-4EF3-93F7-455BF9EA77A8}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{978B4D1D-D7B3-4D60-B993-465FC28718A5}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2905,7 +2905,9 @@
       <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" ht="14.4">
-      <c r="A68" s="6"/>
+      <c r="A68" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B68" s="19" t="s">
         <v>130</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): add LC 20 Valid Parentheses & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{978B4D1D-D7B3-4D60-B993-465FC28718A5}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66B7E2FD-0458-4C1A-BD0D-F45DC47047C8}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2918,7 +2918,9 @@
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" ht="14.4">
-      <c r="A69" s="6"/>
+      <c r="A69" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B69" s="9" t="s">
         <v>132</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): add LC 503 Next Greater Element II & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66B7E2FD-0458-4C1A-BD0D-F45DC47047C8}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DF87A67-1D8A-48A4-9E24-3B4314240418}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2940,7 +2940,9 @@
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="14.4">
-      <c r="A71" s="6"/>
+      <c r="A71" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B71" s="9" t="s">
         <v>135</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): add LC 739 Daily Temperatures & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DF87A67-1D8A-48A4-9E24-3B4314240418}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61F4F1C3-EF19-41F7-8325-5E5239D6ABEF}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2953,7 +2953,9 @@
       <c r="E71" s="13"/>
     </row>
     <row r="72" spans="1:5" ht="14.4">
-      <c r="A72" s="6"/>
+      <c r="A72" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B72" s="9" t="s">
         <v>137</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): add LC 2487 Remove Nodes From Linked List & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61F4F1C3-EF19-41F7-8325-5E5239D6ABEF}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA92C638-431D-4DB1-A82B-ED5E0FC98FFB}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2966,7 +2966,9 @@
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="14.4">
-      <c r="A73" s="6"/>
+      <c r="A73" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B73" s="6" t="s">
         <v>139</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): add LC 1209 Remove All Adjacent Duplicates in String II & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA92C638-431D-4DB1-A82B-ED5E0FC98FFB}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{220B793D-7E83-4EDB-BB0B-1908629DBF1E}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2979,7 +2979,9 @@
       <c r="E73" s="8"/>
     </row>
     <row r="74" spans="1:5" ht="14.4">
-      <c r="A74" s="6"/>
+      <c r="A74" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B74" s="9" t="s">
         <v>141</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): add LC 71 Simplify Path & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{220B793D-7E83-4EDB-BB0B-1908629DBF1E}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AB1DFD3-65E3-4679-88AF-906B0C6EDA0D}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2992,7 +2992,9 @@
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" ht="14.4">
-      <c r="A75" s="6"/>
+      <c r="A75" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B75" s="6" t="s">
         <v>143</v>
       </c>

</xml_diff>

<commit_message>
feat(stack): add LC 402 Remove K Digits & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AB1DFD3-65E3-4679-88AF-906B0C6EDA0D}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F975656-7B1C-41FE-92E7-24EF2B88A91D}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3005,7 +3005,9 @@
       <c r="E75" s="8"/>
     </row>
     <row r="76" spans="1:5" ht="14.4">
-      <c r="A76" s="6"/>
+      <c r="A76" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B76" s="6" t="s">
         <v>145</v>
       </c>

</xml_diff>

<commit_message>
feat(hash-table): create Hash-Table directory, add LC 387 First Unique Character in a String & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F975656-7B1C-41FE-92E7-24EF2B88A91D}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E72A7B9-C320-4D28-8CA3-8390916A44F6}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3027,7 +3027,9 @@
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" ht="14.4">
-      <c r="A78" s="6"/>
+      <c r="A78" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B78" s="9" t="s">
         <v>148</v>
       </c>

</xml_diff>

<commit_message>
feat(hash-table): add LC 1189 Maximum Number of Balloons & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E72A7B9-C320-4D28-8CA3-8390916A44F6}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98327C31-DDEB-4123-B534-495CFBA5A4D5}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3040,7 +3040,9 @@
       <c r="E78" s="8"/>
     </row>
     <row r="79" spans="1:5" ht="14.4">
-      <c r="A79" s="6"/>
+      <c r="A79" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B79" s="9" t="s">
         <v>150</v>
       </c>

</xml_diff>

<commit_message>
feat(hash-table): add LC 409 Longest Palindrome & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98327C31-DDEB-4123-B534-495CFBA5A4D5}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27E18DEA-E639-4F3A-878F-BD3D825C5159}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3053,7 +3053,9 @@
       <c r="E79" s="8"/>
     </row>
     <row r="80" spans="1:5" ht="14.4">
-      <c r="A80" s="6"/>
+      <c r="A80" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B80" s="9" t="s">
         <v>152</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): create Binary-Search directory, add LC 704 Binary Search & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27E18DEA-E639-4F3A-878F-BD3D825C5159}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C9F6CE6-6818-4DAF-A768-8A136C8558BC}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3066,7 +3066,9 @@
       <c r="E80" s="8"/>
     </row>
     <row r="81" spans="1:5" ht="14.4">
-      <c r="A81" s="6"/>
+      <c r="A81" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B81" s="9" t="s">
         <v>154</v>
       </c>
@@ -3086,7 +3088,9 @@
       <c r="E82" s="8"/>
     </row>
     <row r="83" spans="1:5" ht="14.4">
-      <c r="A83" s="6"/>
+      <c r="A83" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B83" s="9" t="s">
         <v>157</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 34 Find First and Last Position of Element in Sorted Array & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C9F6CE6-6818-4DAF-A768-8A136C8558BC}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FB7D5FE-B3FE-4535-B59B-56EB7EB71BB0}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3112,7 +3112,9 @@
       <c r="E84" s="8"/>
     </row>
     <row r="85" spans="1:5" ht="14.4">
-      <c r="A85" s="6"/>
+      <c r="A85" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B85" s="9" t="s">
         <v>161</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 852 Peak Index in a Mountain Array & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FB7D5FE-B3FE-4535-B59B-56EB7EB71BB0}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1D7C89A-508B-49DD-B5D0-B3E4117A7544}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3147,7 +3147,9 @@
       <c r="E87" s="8"/>
     </row>
     <row r="88" spans="1:5" ht="14.4">
-      <c r="A88" s="6"/>
+      <c r="A88" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B88" s="9" t="s">
         <v>167</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 153 Find Minimum in Rotated Sorted Array & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D8D8ED5-0FE8-4730-BA04-91EB13E03607}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74264847-549D-455B-B5ED-BAC056878DA8}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3173,7 +3173,9 @@
       <c r="E89" s="8"/>
     </row>
     <row r="90" spans="1:5" ht="14.4">
-      <c r="A90" s="6"/>
+      <c r="A90" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B90" s="9" t="s">
         <v>171</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 33 Search in Rotated Sorted Array & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74264847-549D-455B-B5ED-BAC056878DA8}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF31F71-D5C5-4CC1-9039-AE4734091B57}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3197,7 +3197,9 @@
       <c r="E91" s="8"/>
     </row>
     <row r="92" spans="1:5" ht="14.4">
-      <c r="A92" s="6"/>
+      <c r="A92" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B92" s="9" t="s">
         <v>175</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 875 Koko Eating Bananas & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF31F71-D5C5-4CC1-9039-AE4734091B57}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F37F9244-1B54-4751-8263-DDF27EF0F3BF}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3210,7 +3210,9 @@
       <c r="E92" s="8"/>
     </row>
     <row r="93" spans="1:5" ht="14.4">
-      <c r="A93" s="6"/>
+      <c r="A93" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B93" s="9" t="s">
         <v>177</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 1482 Minimum Number of Days to Make m Bouquets & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F37F9244-1B54-4751-8263-DDF27EF0F3BF}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{750CE4F6-03E1-4DB8-8851-5533953E9A22}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3223,7 +3223,9 @@
       <c r="E93" s="8"/>
     </row>
     <row r="94" spans="1:5" ht="14.4">
-      <c r="A94" s="6"/>
+      <c r="A94" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B94" s="6" t="s">
         <v>179</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 275 H-Index II & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{750CE4F6-03E1-4DB8-8851-5533953E9A22}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABDBC027-5CF3-4734-B33D-6321E7EB2389}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3247,7 +3247,9 @@
       <c r="E95" s="8"/>
     </row>
     <row r="96" spans="1:5" ht="14.4">
-      <c r="A96" s="6"/>
+      <c r="A96" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B96" s="21" t="s">
         <v>183</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 2226 Maximum Candies Allocated to K Children & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABDBC027-5CF3-4734-B33D-6321E7EB2389}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EB7111F-2CA7-444B-882E-443A601AF749}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3260,7 +3260,9 @@
       <c r="E96" s="8"/>
     </row>
     <row r="97" spans="1:5" ht="14.4">
-      <c r="A97" s="6"/>
+      <c r="A97" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B97" s="6" t="s">
         <v>185</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 1011 Capacity To Ship Packages Within D Days & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EB7111F-2CA7-444B-882E-443A601AF749}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5D8F857-103E-4D2B-A32A-D3F61556E1B8}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3273,7 +3273,9 @@
       <c r="E97" s="8"/>
     </row>
     <row r="98" spans="1:5" ht="14.4">
-      <c r="A98" s="6"/>
+      <c r="A98" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B98" s="6" t="s">
         <v>187</v>
       </c>

</xml_diff>

<commit_message>
feat(binary-search): add LC 410 Split Array Largest Sum & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5D8F857-103E-4D2B-A32A-D3F61556E1B8}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACE22E5A-AFF4-4C5F-A851-9D2896BAED4E}"/>
   <bookViews>
     <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -3297,7 +3297,9 @@
       <c r="E99" s="8"/>
     </row>
     <row r="100" spans="1:5" ht="14.4">
-      <c r="A100" s="6"/>
+      <c r="A100" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B100" s="6" t="s">
         <v>191</v>
       </c>

</xml_diff>